<commit_message>
Added the order function for the gui and made a small change on how summaries function is called
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>868 mm</t>
+          <t>968 mm</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>868 mm</t>
+          <t>968 mm</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>868 mm</t>
+          <t>968 mm</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -572,14 +572,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>450 mm</t>
+          <t>500 mm</t>
         </is>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -590,7 +590,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>890 mm</t>
+          <t>990 mm</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>868 mm</t>
+          <t>968 mm</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>418 mm</t>
+          <t>868 mm</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>570 mm</t>
+          <t>270 mm</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -653,7 +653,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cleat</t>
+          <t>top_panel</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -663,101 +663,112 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>418 mm</t>
+          <t>868 mm</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>80 mm</t>
-        </is>
+          <t>760 mm</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>backstrip</t>
+          <t>side_panel</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>front</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>418 mm</t>
+          <t>760 mm</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>80 mm</t>
-        </is>
+          <t>270 mm</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>masonite</t>
+          <t>backstrip</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>440 mm</t>
+          <t>868 mm</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>730 mm</t>
+          <t>80 mm</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>shelf</t>
+          <t>door</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>all</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>418 mm</t>
+          <t>760 mm</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>560 mm</t>
-        </is>
+          <t>450 mm</t>
+        </is>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bottom_panel</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>front</t>
+          <t>masonite</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>418 mm</t>
+          <t>890 mm</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>270 mm</t>
-        </is>
-      </c>
-      <c r="E14" t="b">
-        <v>1</v>
+          <t>750 mm</t>
+        </is>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -766,35 +777,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>top_panel</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>front</t>
+          <t>shelf</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>418 mm</t>
+          <t>868 mm</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>760 mm</t>
-        </is>
-      </c>
-      <c r="E15" t="b">
-        <v>1</v>
+          <t>260 mm</t>
+        </is>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>side_panel</t>
+          <t>bottom_panel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -804,7 +807,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>760 mm</t>
+          <t>418 mm</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -816,31 +819,31 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>door</t>
+          <t>top_panel</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>front</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>418 mm</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>760 mm</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>450 mm</t>
-        </is>
-      </c>
-      <c r="F17" t="b">
+      <c r="E17" t="b">
         <v>1</v>
       </c>
       <c r="G17" t="n">
@@ -850,75 +853,67 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>masonite</t>
+          <t>backstrip</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>440 mm</t>
+          <t>418 mm</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>750 mm</t>
+          <t>80 mm</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>shelf</t>
+          <t>masonite</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>418 mm</t>
+          <t>440 mm</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>260 mm</t>
+          <t>750 mm</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bottom_panel</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>front</t>
+          <t>shelf</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>568 mm</t>
+          <t>418 mm</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>270 mm</t>
-        </is>
-      </c>
-      <c r="E20" t="b">
-        <v>1</v>
+          <t>260 mm</t>
+        </is>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>top_panel</t>
+          <t>bottom_panel</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -928,12 +923,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>568 mm</t>
+          <t>418 mm</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>760 mm</t>
+          <t>570 mm</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -946,12 +941,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>backstrip</t>
+          <t>cleat</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>front</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>568 mm</t>
+          <t>418 mm</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -976,19 +976,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>760 mm</t>
+          <t>740 mm</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>300 mm</t>
+          <t>450 mm</t>
         </is>
       </c>
       <c r="F23" t="b">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -999,12 +999,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>590 mm</t>
+          <t>440 mm</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>750 mm</t>
+          <t>730 mm</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1019,16 +1019,16 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>568 mm</t>
+          <t>418 mm</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>260 mm</t>
+          <t>560 mm</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>